<commit_message>
changed data files (both)
</commit_message>
<xml_diff>
--- a/data/seln-by-year.xlsx
+++ b/data/seln-by-year.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11207"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jeff.coburn/github/seln_map_timeline/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B64B2ED7-E2F6-254A-87C8-8698814828A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{354E5F12-D0F8-3A45-90D3-1BB93BD27CD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="620" windowWidth="34540" windowHeight="18400" xr2:uid="{47A0ACE4-4E48-47E6-8037-4A624CC7927A}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="43">
   <si>
     <t>Total</t>
   </si>
@@ -165,6 +165,9 @@
   </si>
   <si>
     <t>Washington DC</t>
+  </si>
+  <si>
+    <t>Kansas</t>
   </si>
 </sst>
 </file>
@@ -766,7 +769,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{29D12B53-DAAC-4AAF-981B-E955C199365F}">
-  <dimension ref="A2:W44"/>
+  <dimension ref="A2:W45"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <sheetData>
     <row r="2" spans="1:23" ht="16">
@@ -924,7 +927,7 @@
         <v>1</v>
       </c>
       <c r="W4" s="14">
-        <f t="shared" ref="W4:W42" si="0">SUM(C4:V4)</f>
+        <f t="shared" ref="W4:W43" si="0">SUM(C4:V4)</f>
         <v>1.0833333333333333</v>
       </c>
     </row>
@@ -1559,280 +1562,258 @@
       </c>
     </row>
     <row r="17" spans="1:23">
-      <c r="A17" s="20" t="s">
-        <v>14</v>
-      </c>
-      <c r="B17" s="20"/>
-      <c r="C17" s="15">
-        <v>1</v>
-      </c>
-      <c r="D17" s="16">
-        <v>1</v>
-      </c>
-      <c r="E17" s="16">
-        <v>1</v>
-      </c>
-      <c r="F17" s="16">
-        <v>1</v>
-      </c>
-      <c r="G17" s="16">
-        <v>1</v>
-      </c>
-      <c r="H17" s="16">
-        <v>1</v>
-      </c>
-      <c r="I17" s="16">
-        <v>1</v>
-      </c>
+      <c r="A17" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="B17" s="15"/>
+      <c r="C17" s="15"/>
+      <c r="D17" s="16"/>
+      <c r="E17" s="16"/>
+      <c r="F17" s="16"/>
+      <c r="G17" s="16"/>
+      <c r="H17" s="16"/>
+      <c r="I17" s="16"/>
       <c r="J17" s="16"/>
       <c r="K17" s="16"/>
       <c r="L17" s="16"/>
       <c r="M17" s="18"/>
       <c r="N17" s="18"/>
       <c r="O17" s="18"/>
-      <c r="P17" s="18">
-        <v>1</v>
-      </c>
-      <c r="Q17" s="18">
-        <v>1</v>
-      </c>
-      <c r="R17" s="18">
-        <v>1</v>
-      </c>
-      <c r="S17" s="18">
-        <v>1</v>
-      </c>
-      <c r="T17" s="18">
-        <v>1</v>
-      </c>
-      <c r="U17" s="18">
-        <v>1</v>
-      </c>
+      <c r="P17" s="18"/>
+      <c r="Q17" s="18"/>
+      <c r="R17" s="18"/>
+      <c r="S17" s="18"/>
+      <c r="T17" s="18"/>
+      <c r="U17" s="18"/>
       <c r="V17" s="5">
         <v>1</v>
       </c>
       <c r="W17" s="7">
-        <f t="shared" si="0"/>
+        <f>SUM(C17:V17)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:23">
+      <c r="A18" s="20" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="18" spans="1:23">
-      <c r="A18" s="15" t="s">
+      <c r="B18" s="20"/>
+      <c r="C18" s="15">
+        <v>1</v>
+      </c>
+      <c r="D18" s="16">
+        <v>1</v>
+      </c>
+      <c r="E18" s="16">
+        <v>1</v>
+      </c>
+      <c r="F18" s="16">
+        <v>1</v>
+      </c>
+      <c r="G18" s="16">
+        <v>1</v>
+      </c>
+      <c r="H18" s="16">
+        <v>1</v>
+      </c>
+      <c r="I18" s="16">
+        <v>1</v>
+      </c>
+      <c r="J18" s="16"/>
+      <c r="K18" s="16"/>
+      <c r="L18" s="16"/>
+      <c r="M18" s="18"/>
+      <c r="N18" s="18"/>
+      <c r="O18" s="18"/>
+      <c r="P18" s="18">
+        <v>1</v>
+      </c>
+      <c r="Q18" s="18">
+        <v>1</v>
+      </c>
+      <c r="R18" s="18">
+        <v>1</v>
+      </c>
+      <c r="S18" s="18">
+        <v>1</v>
+      </c>
+      <c r="T18" s="18">
+        <v>1</v>
+      </c>
+      <c r="U18" s="18">
+        <v>1</v>
+      </c>
+      <c r="V18" s="5">
+        <v>1</v>
+      </c>
+      <c r="W18" s="7">
+        <f t="shared" si="0"/>
+        <v>14</v>
+      </c>
+    </row>
+    <row r="19" spans="1:23">
+      <c r="A19" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="B18" s="15"/>
-      <c r="C18" s="15">
-        <v>1</v>
-      </c>
-      <c r="D18" s="16">
-        <v>1</v>
-      </c>
-      <c r="E18" s="16">
-        <v>1</v>
-      </c>
-      <c r="F18" s="16">
-        <v>1</v>
-      </c>
-      <c r="G18" s="16">
-        <v>1</v>
-      </c>
-      <c r="H18" s="16">
-        <v>1</v>
-      </c>
-      <c r="I18" s="16">
-        <v>1</v>
-      </c>
-      <c r="J18" s="16">
-        <v>1</v>
-      </c>
-      <c r="K18" s="16">
-        <v>1</v>
-      </c>
-      <c r="L18" s="16">
-        <v>1</v>
-      </c>
-      <c r="M18" s="18">
-        <v>1</v>
-      </c>
-      <c r="N18" s="18">
-        <v>1</v>
-      </c>
-      <c r="O18" s="18">
-        <v>1</v>
-      </c>
-      <c r="P18" s="18">
-        <v>1</v>
-      </c>
-      <c r="Q18" s="18">
-        <v>1</v>
-      </c>
-      <c r="R18" s="18">
-        <v>1</v>
-      </c>
-      <c r="S18" s="18">
-        <v>1</v>
-      </c>
-      <c r="T18" s="18">
-        <v>1</v>
-      </c>
-      <c r="U18" s="18">
-        <v>1</v>
-      </c>
-      <c r="V18" s="5">
-        <v>1</v>
-      </c>
-      <c r="W18" s="7">
+      <c r="B19" s="15"/>
+      <c r="C19" s="15">
+        <v>1</v>
+      </c>
+      <c r="D19" s="16">
+        <v>1</v>
+      </c>
+      <c r="E19" s="16">
+        <v>1</v>
+      </c>
+      <c r="F19" s="16">
+        <v>1</v>
+      </c>
+      <c r="G19" s="16">
+        <v>1</v>
+      </c>
+      <c r="H19" s="16">
+        <v>1</v>
+      </c>
+      <c r="I19" s="16">
+        <v>1</v>
+      </c>
+      <c r="J19" s="16">
+        <v>1</v>
+      </c>
+      <c r="K19" s="16">
+        <v>1</v>
+      </c>
+      <c r="L19" s="16">
+        <v>1</v>
+      </c>
+      <c r="M19" s="18">
+        <v>1</v>
+      </c>
+      <c r="N19" s="18">
+        <v>1</v>
+      </c>
+      <c r="O19" s="18">
+        <v>1</v>
+      </c>
+      <c r="P19" s="18">
+        <v>1</v>
+      </c>
+      <c r="Q19" s="18">
+        <v>1</v>
+      </c>
+      <c r="R19" s="18">
+        <v>1</v>
+      </c>
+      <c r="S19" s="18">
+        <v>1</v>
+      </c>
+      <c r="T19" s="18">
+        <v>1</v>
+      </c>
+      <c r="U19" s="18">
+        <v>1</v>
+      </c>
+      <c r="V19" s="5">
+        <v>1</v>
+      </c>
+      <c r="W19" s="7">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
     </row>
-    <row r="19" spans="1:23">
-      <c r="A19" s="21" t="s">
+    <row r="20" spans="1:23">
+      <c r="A20" s="21" t="s">
         <v>40</v>
       </c>
-      <c r="B19" s="21"/>
-      <c r="C19" s="21">
-        <v>1</v>
-      </c>
-      <c r="D19" s="22">
-        <v>1</v>
-      </c>
-      <c r="E19" s="22">
-        <v>1</v>
-      </c>
-      <c r="F19" s="22">
-        <v>1</v>
-      </c>
-      <c r="G19" s="22">
-        <v>1</v>
-      </c>
-      <c r="H19" s="22">
-        <v>1</v>
-      </c>
-      <c r="I19" s="22">
-        <v>1</v>
-      </c>
-      <c r="J19" s="22">
-        <v>1</v>
-      </c>
-      <c r="K19" s="22">
-        <v>1</v>
-      </c>
-      <c r="L19" s="22">
-        <v>1</v>
-      </c>
-      <c r="M19" s="23">
-        <v>1</v>
-      </c>
-      <c r="N19" s="23">
-        <v>1</v>
-      </c>
-      <c r="O19" s="23">
-        <v>1</v>
-      </c>
-      <c r="P19" s="23">
-        <v>1</v>
-      </c>
-      <c r="Q19" s="23">
-        <v>1</v>
-      </c>
-      <c r="R19" s="23">
-        <v>1</v>
-      </c>
-      <c r="S19" s="23">
-        <v>1</v>
-      </c>
-      <c r="T19" s="23">
-        <v>1</v>
-      </c>
-      <c r="U19" s="23">
-        <v>1</v>
-      </c>
-      <c r="V19" s="24">
-        <v>1</v>
-      </c>
-      <c r="W19" s="25">
+      <c r="B20" s="21"/>
+      <c r="C20" s="21">
+        <v>1</v>
+      </c>
+      <c r="D20" s="22">
+        <v>1</v>
+      </c>
+      <c r="E20" s="22">
+        <v>1</v>
+      </c>
+      <c r="F20" s="22">
+        <v>1</v>
+      </c>
+      <c r="G20" s="22">
+        <v>1</v>
+      </c>
+      <c r="H20" s="22">
+        <v>1</v>
+      </c>
+      <c r="I20" s="22">
+        <v>1</v>
+      </c>
+      <c r="J20" s="22">
+        <v>1</v>
+      </c>
+      <c r="K20" s="22">
+        <v>1</v>
+      </c>
+      <c r="L20" s="22">
+        <v>1</v>
+      </c>
+      <c r="M20" s="23">
+        <v>1</v>
+      </c>
+      <c r="N20" s="23">
+        <v>1</v>
+      </c>
+      <c r="O20" s="23">
+        <v>1</v>
+      </c>
+      <c r="P20" s="23">
+        <v>1</v>
+      </c>
+      <c r="Q20" s="23">
+        <v>1</v>
+      </c>
+      <c r="R20" s="23">
+        <v>1</v>
+      </c>
+      <c r="S20" s="23">
+        <v>1</v>
+      </c>
+      <c r="T20" s="23">
+        <v>1</v>
+      </c>
+      <c r="U20" s="23">
+        <v>1</v>
+      </c>
+      <c r="V20" s="24">
+        <v>1</v>
+      </c>
+      <c r="W20" s="25">
         <f t="shared" si="0"/>
         <v>20</v>
-      </c>
-    </row>
-    <row r="20" spans="1:23">
-      <c r="A20" s="15" t="s">
-        <v>16</v>
-      </c>
-      <c r="B20" s="15"/>
-      <c r="C20" s="15"/>
-      <c r="D20" s="16"/>
-      <c r="E20" s="16"/>
-      <c r="F20" s="16">
-        <v>1</v>
-      </c>
-      <c r="G20" s="16">
-        <v>1</v>
-      </c>
-      <c r="H20" s="16">
-        <v>1</v>
-      </c>
-      <c r="I20" s="16">
-        <v>1</v>
-      </c>
-      <c r="J20" s="16">
-        <v>1</v>
-      </c>
-      <c r="K20" s="16">
-        <v>1</v>
-      </c>
-      <c r="L20" s="16">
-        <v>1</v>
-      </c>
-      <c r="M20" s="18">
-        <v>1</v>
-      </c>
-      <c r="N20" s="18">
-        <v>1</v>
-      </c>
-      <c r="O20" s="18">
-        <v>1</v>
-      </c>
-      <c r="P20" s="18">
-        <v>1</v>
-      </c>
-      <c r="Q20" s="18">
-        <v>1</v>
-      </c>
-      <c r="R20" s="18">
-        <v>1</v>
-      </c>
-      <c r="S20" s="18">
-        <v>1</v>
-      </c>
-      <c r="T20" s="18">
-        <v>1</v>
-      </c>
-      <c r="U20" s="18">
-        <v>1</v>
-      </c>
-      <c r="V20" s="5">
-        <v>1</v>
-      </c>
-      <c r="W20" s="26">
-        <f t="shared" si="0"/>
-        <v>17</v>
       </c>
     </row>
     <row r="21" spans="1:23">
       <c r="A21" s="15" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B21" s="15"/>
       <c r="C21" s="15"/>
       <c r="D21" s="16"/>
       <c r="E21" s="16"/>
-      <c r="F21" s="16"/>
-      <c r="G21" s="16"/>
-      <c r="H21" s="16"/>
-      <c r="I21" s="16"/>
-      <c r="J21" s="16"/>
+      <c r="F21" s="16">
+        <v>1</v>
+      </c>
+      <c r="G21" s="16">
+        <v>1</v>
+      </c>
+      <c r="H21" s="16">
+        <v>1</v>
+      </c>
+      <c r="I21" s="16">
+        <v>1</v>
+      </c>
+      <c r="J21" s="16">
+        <v>1</v>
+      </c>
       <c r="K21" s="16">
         <v>1</v>
       </c>
@@ -1851,9 +1832,11 @@
       <c r="P21" s="18">
         <v>1</v>
       </c>
-      <c r="Q21" s="18"/>
+      <c r="Q21" s="18">
+        <v>1</v>
+      </c>
       <c r="R21" s="18">
-        <v>0.75</v>
+        <v>1</v>
       </c>
       <c r="S21" s="18">
         <v>1</v>
@@ -1869,34 +1852,22 @@
       </c>
       <c r="W21" s="26">
         <f t="shared" si="0"/>
-        <v>10.75</v>
+        <v>17</v>
       </c>
     </row>
     <row r="22" spans="1:23">
       <c r="A22" s="15" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B22" s="15"/>
       <c r="C22" s="15"/>
       <c r="D22" s="16"/>
-      <c r="E22" s="16">
-        <v>1</v>
-      </c>
-      <c r="F22" s="16">
-        <v>1</v>
-      </c>
-      <c r="G22" s="16">
-        <v>1</v>
-      </c>
-      <c r="H22" s="16">
-        <v>1</v>
-      </c>
-      <c r="I22" s="16">
-        <v>1</v>
-      </c>
-      <c r="J22" s="16">
-        <v>1</v>
-      </c>
+      <c r="E22" s="16"/>
+      <c r="F22" s="16"/>
+      <c r="G22" s="16"/>
+      <c r="H22" s="16"/>
+      <c r="I22" s="16"/>
+      <c r="J22" s="16"/>
       <c r="K22" s="16">
         <v>1</v>
       </c>
@@ -1915,11 +1886,9 @@
       <c r="P22" s="18">
         <v>1</v>
       </c>
-      <c r="Q22" s="18">
-        <v>1</v>
-      </c>
+      <c r="Q22" s="18"/>
       <c r="R22" s="18">
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="S22" s="18">
         <v>1</v>
@@ -1935,18 +1904,22 @@
       </c>
       <c r="W22" s="26">
         <f t="shared" si="0"/>
+        <v>10.75</v>
+      </c>
+    </row>
+    <row r="23" spans="1:23">
+      <c r="A23" s="15" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="23" spans="1:23">
-      <c r="A23" s="20" t="s">
-        <v>39</v>
-      </c>
-      <c r="B23" s="20"/>
+      <c r="B23" s="15"/>
       <c r="C23" s="15"/>
       <c r="D23" s="16"/>
-      <c r="E23" s="16"/>
-      <c r="F23" s="16"/>
+      <c r="E23" s="16">
+        <v>1</v>
+      </c>
+      <c r="F23" s="16">
+        <v>1</v>
+      </c>
       <c r="G23" s="16">
         <v>1</v>
       </c>
@@ -1962,32 +1935,56 @@
       <c r="K23" s="16">
         <v>1</v>
       </c>
-      <c r="L23" s="16"/>
-      <c r="M23" s="18"/>
-      <c r="N23" s="18"/>
-      <c r="O23" s="18"/>
-      <c r="P23" s="18"/>
-      <c r="Q23" s="18"/>
-      <c r="R23" s="18"/>
-      <c r="S23" s="18"/>
-      <c r="T23" s="18"/>
-      <c r="U23" s="18"/>
-      <c r="V23" s="5"/>
+      <c r="L23" s="16">
+        <v>1</v>
+      </c>
+      <c r="M23" s="18">
+        <v>1</v>
+      </c>
+      <c r="N23" s="18">
+        <v>1</v>
+      </c>
+      <c r="O23" s="18">
+        <v>1</v>
+      </c>
+      <c r="P23" s="18">
+        <v>1</v>
+      </c>
+      <c r="Q23" s="18">
+        <v>1</v>
+      </c>
+      <c r="R23" s="18">
+        <v>1</v>
+      </c>
+      <c r="S23" s="18">
+        <v>1</v>
+      </c>
+      <c r="T23" s="18">
+        <v>1</v>
+      </c>
+      <c r="U23" s="18">
+        <v>1</v>
+      </c>
+      <c r="V23" s="5">
+        <v>1</v>
+      </c>
       <c r="W23" s="26">
         <f t="shared" si="0"/>
-        <v>5</v>
+        <v>18</v>
       </c>
     </row>
     <row r="24" spans="1:23">
-      <c r="A24" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="B24" s="15"/>
+      <c r="A24" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="B24" s="20"/>
       <c r="C24" s="15"/>
       <c r="D24" s="16"/>
       <c r="E24" s="16"/>
       <c r="F24" s="16"/>
-      <c r="G24" s="16"/>
+      <c r="G24" s="16">
+        <v>1</v>
+      </c>
       <c r="H24" s="16">
         <v>1</v>
       </c>
@@ -2000,52 +1997,32 @@
       <c r="K24" s="16">
         <v>1</v>
       </c>
-      <c r="L24" s="16">
-        <v>1</v>
-      </c>
+      <c r="L24" s="16"/>
       <c r="M24" s="18"/>
       <c r="N24" s="18"/>
       <c r="O24" s="18"/>
       <c r="P24" s="18"/>
       <c r="Q24" s="18"/>
       <c r="R24" s="18"/>
-      <c r="S24" s="18">
-        <v>0.75</v>
-      </c>
-      <c r="T24" s="18">
-        <v>1</v>
-      </c>
-      <c r="U24" s="18">
-        <v>1</v>
-      </c>
-      <c r="V24" s="5">
-        <v>1</v>
-      </c>
+      <c r="S24" s="18"/>
+      <c r="T24" s="18"/>
+      <c r="U24" s="18"/>
+      <c r="V24" s="5"/>
       <c r="W24" s="26">
         <f t="shared" si="0"/>
-        <v>8.75</v>
+        <v>5</v>
       </c>
     </row>
     <row r="25" spans="1:23">
       <c r="A25" s="15" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B25" s="15"/>
-      <c r="C25" s="15">
-        <v>1</v>
-      </c>
-      <c r="D25" s="16">
-        <v>1</v>
-      </c>
-      <c r="E25" s="16">
-        <v>1</v>
-      </c>
-      <c r="F25" s="16">
-        <v>1</v>
-      </c>
-      <c r="G25" s="16">
-        <v>1</v>
-      </c>
+      <c r="C25" s="15"/>
+      <c r="D25" s="16"/>
+      <c r="E25" s="16"/>
+      <c r="F25" s="16"/>
+      <c r="G25" s="16"/>
       <c r="H25" s="16">
         <v>1</v>
       </c>
@@ -2061,26 +2038,14 @@
       <c r="L25" s="16">
         <v>1</v>
       </c>
-      <c r="M25" s="18">
-        <v>1</v>
-      </c>
-      <c r="N25" s="18">
-        <v>1</v>
-      </c>
-      <c r="O25" s="18">
-        <v>1</v>
-      </c>
-      <c r="P25" s="18">
-        <v>1</v>
-      </c>
-      <c r="Q25" s="18">
-        <v>1</v>
-      </c>
-      <c r="R25" s="18">
-        <v>1</v>
-      </c>
+      <c r="M25" s="18"/>
+      <c r="N25" s="18"/>
+      <c r="O25" s="18"/>
+      <c r="P25" s="18"/>
+      <c r="Q25" s="18"/>
+      <c r="R25" s="18"/>
       <c r="S25" s="18">
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="T25" s="18">
         <v>1</v>
@@ -2093,21 +2058,35 @@
       </c>
       <c r="W25" s="26">
         <f t="shared" si="0"/>
-        <v>20</v>
+        <v>8.75</v>
       </c>
     </row>
     <row r="26" spans="1:23">
       <c r="A26" s="15" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B26" s="15"/>
-      <c r="C26" s="15"/>
-      <c r="D26" s="16"/>
-      <c r="E26" s="16"/>
-      <c r="F26" s="16"/>
-      <c r="G26" s="16"/>
-      <c r="H26" s="16"/>
-      <c r="I26" s="16"/>
+      <c r="C26" s="15">
+        <v>1</v>
+      </c>
+      <c r="D26" s="16">
+        <v>1</v>
+      </c>
+      <c r="E26" s="16">
+        <v>1</v>
+      </c>
+      <c r="F26" s="16">
+        <v>1</v>
+      </c>
+      <c r="G26" s="16">
+        <v>1</v>
+      </c>
+      <c r="H26" s="16">
+        <v>1</v>
+      </c>
+      <c r="I26" s="16">
+        <v>1</v>
+      </c>
       <c r="J26" s="16">
         <v>1</v>
       </c>
@@ -2149,31 +2128,21 @@
       </c>
       <c r="W26" s="26">
         <f t="shared" si="0"/>
-        <v>13</v>
+        <v>20</v>
       </c>
     </row>
     <row r="27" spans="1:23">
       <c r="A27" s="15" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B27" s="15"/>
       <c r="C27" s="15"/>
       <c r="D27" s="16"/>
-      <c r="E27" s="16">
-        <v>1</v>
-      </c>
-      <c r="F27" s="16">
-        <v>1</v>
-      </c>
-      <c r="G27" s="16">
-        <v>1</v>
-      </c>
-      <c r="H27" s="16">
-        <v>1</v>
-      </c>
-      <c r="I27" s="16">
-        <v>1</v>
-      </c>
+      <c r="E27" s="16"/>
+      <c r="F27" s="16"/>
+      <c r="G27" s="16"/>
+      <c r="H27" s="16"/>
+      <c r="I27" s="16"/>
       <c r="J27" s="16">
         <v>1</v>
       </c>
@@ -2186,30 +2155,54 @@
       <c r="M27" s="18">
         <v>1</v>
       </c>
-      <c r="N27" s="18"/>
-      <c r="O27" s="18"/>
-      <c r="P27" s="18"/>
-      <c r="Q27" s="18"/>
-      <c r="R27" s="18"/>
-      <c r="S27" s="18"/>
-      <c r="T27" s="18"/>
-      <c r="U27" s="18"/>
-      <c r="V27" s="5"/>
+      <c r="N27" s="18">
+        <v>1</v>
+      </c>
+      <c r="O27" s="18">
+        <v>1</v>
+      </c>
+      <c r="P27" s="18">
+        <v>1</v>
+      </c>
+      <c r="Q27" s="18">
+        <v>1</v>
+      </c>
+      <c r="R27" s="18">
+        <v>1</v>
+      </c>
+      <c r="S27" s="18">
+        <v>1</v>
+      </c>
+      <c r="T27" s="18">
+        <v>1</v>
+      </c>
+      <c r="U27" s="18">
+        <v>1</v>
+      </c>
+      <c r="V27" s="5">
+        <v>1</v>
+      </c>
       <c r="W27" s="26">
         <f t="shared" si="0"/>
-        <v>9</v>
+        <v>13</v>
       </c>
     </row>
     <row r="28" spans="1:23">
-      <c r="A28" s="20" t="s">
-        <v>23</v>
-      </c>
-      <c r="B28" s="20"/>
+      <c r="A28" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="B28" s="15"/>
       <c r="C28" s="15"/>
       <c r="D28" s="16"/>
-      <c r="E28" s="16"/>
-      <c r="F28" s="16"/>
-      <c r="G28" s="16"/>
+      <c r="E28" s="16">
+        <v>1</v>
+      </c>
+      <c r="F28" s="16">
+        <v>1</v>
+      </c>
+      <c r="G28" s="16">
+        <v>1</v>
+      </c>
       <c r="H28" s="16">
         <v>1</v>
       </c>
@@ -2222,34 +2215,31 @@
       <c r="K28" s="16">
         <v>1</v>
       </c>
-      <c r="L28" s="16"/>
-      <c r="M28" s="18"/>
+      <c r="L28" s="16">
+        <v>1</v>
+      </c>
+      <c r="M28" s="18">
+        <v>1</v>
+      </c>
       <c r="N28" s="18"/>
       <c r="O28" s="18"/>
       <c r="P28" s="18"/>
       <c r="Q28" s="18"/>
       <c r="R28" s="18"/>
       <c r="S28" s="18"/>
-      <c r="T28" s="18">
-        <f>11/12</f>
-        <v>0.91666666666666663</v>
-      </c>
-      <c r="U28" s="18">
-        <v>1</v>
-      </c>
-      <c r="V28" s="5">
-        <v>1</v>
-      </c>
+      <c r="T28" s="18"/>
+      <c r="U28" s="18"/>
+      <c r="V28" s="5"/>
       <c r="W28" s="26">
         <f t="shared" si="0"/>
-        <v>6.916666666666667</v>
+        <v>9</v>
       </c>
     </row>
     <row r="29" spans="1:23">
-      <c r="A29" s="15" t="s">
-        <v>24</v>
-      </c>
-      <c r="B29" s="15"/>
+      <c r="A29" s="20" t="s">
+        <v>23</v>
+      </c>
+      <c r="B29" s="20"/>
       <c r="C29" s="15"/>
       <c r="D29" s="16"/>
       <c r="E29" s="16"/>
@@ -2267,32 +2257,17 @@
       <c r="K29" s="16">
         <v>1</v>
       </c>
-      <c r="L29" s="16">
-        <v>1</v>
-      </c>
-      <c r="M29" s="18">
-        <v>1</v>
-      </c>
-      <c r="N29" s="18">
-        <v>1</v>
-      </c>
-      <c r="O29" s="18">
-        <v>1</v>
-      </c>
-      <c r="P29" s="18">
-        <v>1</v>
-      </c>
-      <c r="Q29" s="18">
-        <v>1</v>
-      </c>
-      <c r="R29" s="18">
-        <v>1</v>
-      </c>
-      <c r="S29" s="18">
-        <v>1</v>
-      </c>
+      <c r="L29" s="16"/>
+      <c r="M29" s="18"/>
+      <c r="N29" s="18"/>
+      <c r="O29" s="18"/>
+      <c r="P29" s="18"/>
+      <c r="Q29" s="18"/>
+      <c r="R29" s="18"/>
+      <c r="S29" s="18"/>
       <c r="T29" s="18">
-        <v>1</v>
+        <f>11/12</f>
+        <v>0.91666666666666663</v>
       </c>
       <c r="U29" s="18">
         <v>1</v>
@@ -2302,12 +2277,12 @@
       </c>
       <c r="W29" s="26">
         <f t="shared" si="0"/>
-        <v>15</v>
+        <v>6.916666666666667</v>
       </c>
     </row>
     <row r="30" spans="1:23">
       <c r="A30" s="15" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B30" s="15"/>
       <c r="C30" s="15"/>
@@ -2367,26 +2342,20 @@
     </row>
     <row r="31" spans="1:23">
       <c r="A31" s="15" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B31" s="15"/>
-      <c r="C31" s="15">
-        <v>1</v>
-      </c>
-      <c r="D31" s="16">
-        <v>1</v>
-      </c>
-      <c r="E31" s="16">
-        <v>1</v>
-      </c>
-      <c r="F31" s="16">
-        <v>1</v>
-      </c>
-      <c r="G31" s="16">
-        <v>1</v>
-      </c>
-      <c r="H31" s="16"/>
-      <c r="I31" s="16"/>
+      <c r="C31" s="15"/>
+      <c r="D31" s="16"/>
+      <c r="E31" s="16"/>
+      <c r="F31" s="16"/>
+      <c r="G31" s="16"/>
+      <c r="H31" s="16">
+        <v>1</v>
+      </c>
+      <c r="I31" s="16">
+        <v>1</v>
+      </c>
       <c r="J31" s="16">
         <v>1</v>
       </c>
@@ -2428,12 +2397,12 @@
       </c>
       <c r="W31" s="26">
         <f t="shared" si="0"/>
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="32" spans="1:23">
       <c r="A32" s="15" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B32" s="15"/>
       <c r="C32" s="15">
@@ -2452,9 +2421,7 @@
         <v>1</v>
       </c>
       <c r="H32" s="16"/>
-      <c r="I32" s="16">
-        <v>1</v>
-      </c>
+      <c r="I32" s="16"/>
       <c r="J32" s="16">
         <v>1</v>
       </c>
@@ -2473,30 +2440,56 @@
       <c r="O32" s="18">
         <v>1</v>
       </c>
-      <c r="P32" s="18"/>
-      <c r="Q32" s="18"/>
-      <c r="R32" s="18"/>
-      <c r="S32" s="18"/>
-      <c r="T32" s="18"/>
-      <c r="U32" s="18"/>
-      <c r="V32" s="5"/>
+      <c r="P32" s="18">
+        <v>1</v>
+      </c>
+      <c r="Q32" s="18">
+        <v>1</v>
+      </c>
+      <c r="R32" s="18">
+        <v>1</v>
+      </c>
+      <c r="S32" s="18">
+        <v>1</v>
+      </c>
+      <c r="T32" s="18">
+        <v>1</v>
+      </c>
+      <c r="U32" s="18">
+        <v>1</v>
+      </c>
+      <c r="V32" s="5">
+        <v>1</v>
+      </c>
       <c r="W32" s="26">
         <f t="shared" si="0"/>
-        <v>12</v>
+        <v>18</v>
       </c>
     </row>
     <row r="33" spans="1:23">
       <c r="A33" s="15" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B33" s="15"/>
-      <c r="C33" s="15"/>
-      <c r="D33" s="16"/>
-      <c r="E33" s="16"/>
-      <c r="F33" s="16"/>
-      <c r="G33" s="16"/>
+      <c r="C33" s="15">
+        <v>1</v>
+      </c>
+      <c r="D33" s="16">
+        <v>1</v>
+      </c>
+      <c r="E33" s="16">
+        <v>1</v>
+      </c>
+      <c r="F33" s="16">
+        <v>1</v>
+      </c>
+      <c r="G33" s="16">
+        <v>1</v>
+      </c>
       <c r="H33" s="16"/>
-      <c r="I33" s="16"/>
+      <c r="I33" s="16">
+        <v>1</v>
+      </c>
       <c r="J33" s="16">
         <v>1</v>
       </c>
@@ -2515,149 +2508,121 @@
       <c r="O33" s="18">
         <v>1</v>
       </c>
-      <c r="P33" s="18">
-        <v>1</v>
-      </c>
-      <c r="Q33" s="18">
-        <v>1</v>
-      </c>
-      <c r="R33" s="18">
-        <v>1</v>
-      </c>
-      <c r="S33" s="18">
-        <v>1</v>
-      </c>
-      <c r="T33" s="18">
-        <v>1</v>
-      </c>
-      <c r="U33" s="18">
-        <v>1</v>
-      </c>
-      <c r="V33" s="5">
-        <v>1</v>
-      </c>
+      <c r="P33" s="18"/>
+      <c r="Q33" s="18"/>
+      <c r="R33" s="18"/>
+      <c r="S33" s="18"/>
+      <c r="T33" s="18"/>
+      <c r="U33" s="18"/>
+      <c r="V33" s="5"/>
       <c r="W33" s="26">
         <f t="shared" si="0"/>
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="34" spans="1:23">
       <c r="A34" s="15" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B34" s="15"/>
-      <c r="C34" s="15">
-        <v>1</v>
-      </c>
-      <c r="D34" s="16">
-        <v>1</v>
-      </c>
-      <c r="E34" s="16">
-        <v>1</v>
-      </c>
+      <c r="C34" s="15"/>
+      <c r="D34" s="16"/>
+      <c r="E34" s="16"/>
       <c r="F34" s="16"/>
       <c r="G34" s="16"/>
       <c r="H34" s="16"/>
       <c r="I34" s="16"/>
-      <c r="J34" s="16"/>
-      <c r="K34" s="16"/>
-      <c r="L34" s="16"/>
-      <c r="M34" s="18"/>
-      <c r="N34" s="18"/>
-      <c r="O34" s="18"/>
-      <c r="P34" s="18"/>
-      <c r="Q34" s="18"/>
-      <c r="R34" s="18"/>
-      <c r="S34" s="18"/>
-      <c r="T34" s="18"/>
-      <c r="U34" s="18"/>
-      <c r="V34" s="5"/>
+      <c r="J34" s="16">
+        <v>1</v>
+      </c>
+      <c r="K34" s="16">
+        <v>1</v>
+      </c>
+      <c r="L34" s="16">
+        <v>1</v>
+      </c>
+      <c r="M34" s="18">
+        <v>1</v>
+      </c>
+      <c r="N34" s="18">
+        <v>1</v>
+      </c>
+      <c r="O34" s="18">
+        <v>1</v>
+      </c>
+      <c r="P34" s="18">
+        <v>1</v>
+      </c>
+      <c r="Q34" s="18">
+        <v>1</v>
+      </c>
+      <c r="R34" s="18">
+        <v>1</v>
+      </c>
+      <c r="S34" s="18">
+        <v>1</v>
+      </c>
+      <c r="T34" s="18">
+        <v>1</v>
+      </c>
+      <c r="U34" s="18">
+        <v>1</v>
+      </c>
+      <c r="V34" s="5">
+        <v>1</v>
+      </c>
       <c r="W34" s="26">
         <f t="shared" si="0"/>
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="35" spans="1:23">
       <c r="A35" s="15" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B35" s="15"/>
-      <c r="C35" s="15"/>
-      <c r="D35" s="16"/>
-      <c r="E35" s="16"/>
+      <c r="C35" s="15">
+        <v>1</v>
+      </c>
+      <c r="D35" s="16">
+        <v>1</v>
+      </c>
+      <c r="E35" s="16">
+        <v>1</v>
+      </c>
       <c r="F35" s="16"/>
       <c r="G35" s="16"/>
       <c r="H35" s="16"/>
-      <c r="I35" s="16">
-        <v>1</v>
-      </c>
-      <c r="J35" s="16">
-        <v>1</v>
-      </c>
-      <c r="K35" s="16">
-        <v>1</v>
-      </c>
-      <c r="L35" s="16">
-        <v>1</v>
-      </c>
-      <c r="M35" s="18">
-        <v>1</v>
-      </c>
-      <c r="N35" s="18">
-        <v>1</v>
-      </c>
-      <c r="O35" s="18">
-        <v>1</v>
-      </c>
-      <c r="P35" s="18">
-        <v>1</v>
-      </c>
-      <c r="Q35" s="18">
-        <v>1</v>
-      </c>
-      <c r="R35" s="18">
-        <v>1</v>
-      </c>
-      <c r="S35" s="18">
-        <v>1</v>
-      </c>
-      <c r="T35" s="18">
-        <v>1</v>
-      </c>
-      <c r="U35" s="18">
-        <v>1</v>
-      </c>
-      <c r="V35" s="5">
-        <v>1</v>
-      </c>
+      <c r="I35" s="16"/>
+      <c r="J35" s="16"/>
+      <c r="K35" s="16"/>
+      <c r="L35" s="16"/>
+      <c r="M35" s="18"/>
+      <c r="N35" s="18"/>
+      <c r="O35" s="18"/>
+      <c r="P35" s="18"/>
+      <c r="Q35" s="18"/>
+      <c r="R35" s="18"/>
+      <c r="S35" s="18"/>
+      <c r="T35" s="18"/>
+      <c r="U35" s="18"/>
+      <c r="V35" s="5"/>
       <c r="W35" s="26">
         <f t="shared" si="0"/>
-        <v>14</v>
+        <v>3</v>
       </c>
     </row>
     <row r="36" spans="1:23">
       <c r="A36" s="15" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B36" s="15"/>
-      <c r="C36" s="15">
-        <v>1</v>
-      </c>
-      <c r="D36" s="16">
-        <v>1</v>
-      </c>
-      <c r="E36" s="16">
-        <v>1</v>
-      </c>
-      <c r="F36" s="16">
-        <v>1</v>
-      </c>
-      <c r="G36" s="16">
-        <v>1</v>
-      </c>
-      <c r="H36" s="16">
-        <v>1</v>
-      </c>
+      <c r="C36" s="15"/>
+      <c r="D36" s="16"/>
+      <c r="E36" s="16"/>
+      <c r="F36" s="16"/>
+      <c r="G36" s="16"/>
+      <c r="H36" s="16"/>
       <c r="I36" s="16">
         <v>1</v>
       </c>
@@ -2702,26 +2667,50 @@
       </c>
       <c r="W36" s="26">
         <f t="shared" si="0"/>
-        <v>20</v>
+        <v>14</v>
       </c>
     </row>
     <row r="37" spans="1:23">
       <c r="A37" s="15" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B37" s="15"/>
-      <c r="C37" s="15"/>
-      <c r="D37" s="16"/>
-      <c r="E37" s="16"/>
-      <c r="F37" s="16"/>
-      <c r="G37" s="16"/>
-      <c r="H37" s="16"/>
-      <c r="I37" s="16"/>
-      <c r="J37" s="16"/>
-      <c r="K37" s="16"/>
-      <c r="L37" s="16"/>
-      <c r="M37" s="18"/>
-      <c r="N37" s="18"/>
+      <c r="C37" s="15">
+        <v>1</v>
+      </c>
+      <c r="D37" s="16">
+        <v>1</v>
+      </c>
+      <c r="E37" s="16">
+        <v>1</v>
+      </c>
+      <c r="F37" s="16">
+        <v>1</v>
+      </c>
+      <c r="G37" s="16">
+        <v>1</v>
+      </c>
+      <c r="H37" s="16">
+        <v>1</v>
+      </c>
+      <c r="I37" s="16">
+        <v>1</v>
+      </c>
+      <c r="J37" s="16">
+        <v>1</v>
+      </c>
+      <c r="K37" s="16">
+        <v>1</v>
+      </c>
+      <c r="L37" s="16">
+        <v>1</v>
+      </c>
+      <c r="M37" s="18">
+        <v>1</v>
+      </c>
+      <c r="N37" s="18">
+        <v>1</v>
+      </c>
       <c r="O37" s="18">
         <v>1</v>
       </c>
@@ -2748,44 +2737,26 @@
       </c>
       <c r="W37" s="26">
         <f t="shared" si="0"/>
-        <v>8</v>
+        <v>20</v>
       </c>
     </row>
     <row r="38" spans="1:23">
       <c r="A38" s="15" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B38" s="15"/>
       <c r="C38" s="15"/>
       <c r="D38" s="16"/>
       <c r="E38" s="16"/>
-      <c r="F38" s="16">
-        <v>1</v>
-      </c>
-      <c r="G38" s="16">
-        <v>1</v>
-      </c>
-      <c r="H38" s="16">
-        <v>1</v>
-      </c>
-      <c r="I38" s="16">
-        <v>1</v>
-      </c>
-      <c r="J38" s="16">
-        <v>1</v>
-      </c>
-      <c r="K38" s="16">
-        <v>1</v>
-      </c>
-      <c r="L38" s="16">
-        <v>1</v>
-      </c>
-      <c r="M38" s="18">
-        <v>1</v>
-      </c>
-      <c r="N38" s="18">
-        <v>1</v>
-      </c>
+      <c r="F38" s="16"/>
+      <c r="G38" s="16"/>
+      <c r="H38" s="16"/>
+      <c r="I38" s="16"/>
+      <c r="J38" s="16"/>
+      <c r="K38" s="16"/>
+      <c r="L38" s="16"/>
+      <c r="M38" s="18"/>
+      <c r="N38" s="18"/>
       <c r="O38" s="18">
         <v>1</v>
       </c>
@@ -2812,82 +2783,76 @@
       </c>
       <c r="W38" s="26">
         <f t="shared" si="0"/>
-        <v>17</v>
+        <v>8</v>
       </c>
     </row>
     <row r="39" spans="1:23">
       <c r="A39" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="B39" s="15"/>
+      <c r="C39" s="15"/>
+      <c r="D39" s="16"/>
+      <c r="E39" s="16"/>
+      <c r="F39" s="16">
+        <v>1</v>
+      </c>
+      <c r="G39" s="16">
+        <v>1</v>
+      </c>
+      <c r="H39" s="16">
+        <v>1</v>
+      </c>
+      <c r="I39" s="16">
+        <v>1</v>
+      </c>
+      <c r="J39" s="16">
+        <v>1</v>
+      </c>
+      <c r="K39" s="16">
+        <v>1</v>
+      </c>
+      <c r="L39" s="16">
+        <v>1</v>
+      </c>
+      <c r="M39" s="18">
+        <v>1</v>
+      </c>
+      <c r="N39" s="18">
+        <v>1</v>
+      </c>
+      <c r="O39" s="18">
+        <v>1</v>
+      </c>
+      <c r="P39" s="18">
+        <v>1</v>
+      </c>
+      <c r="Q39" s="18">
+        <v>1</v>
+      </c>
+      <c r="R39" s="18">
+        <v>1</v>
+      </c>
+      <c r="S39" s="18">
+        <v>1</v>
+      </c>
+      <c r="T39" s="18">
+        <v>1</v>
+      </c>
+      <c r="U39" s="18">
+        <v>1</v>
+      </c>
+      <c r="V39" s="5">
+        <v>1</v>
+      </c>
+      <c r="W39" s="26">
+        <f t="shared" si="0"/>
+        <v>17</v>
+      </c>
+    </row>
+    <row r="40" spans="1:23">
+      <c r="A40" s="15" t="s">
         <v>34</v>
-      </c>
-      <c r="B39" s="15"/>
-      <c r="C39" s="15">
-        <v>1</v>
-      </c>
-      <c r="D39" s="16">
-        <v>1</v>
-      </c>
-      <c r="E39" s="16">
-        <v>1</v>
-      </c>
-      <c r="F39" s="16">
-        <v>1</v>
-      </c>
-      <c r="G39" s="16">
-        <v>1</v>
-      </c>
-      <c r="H39" s="16">
-        <v>1</v>
-      </c>
-      <c r="I39" s="16">
-        <v>1</v>
-      </c>
-      <c r="J39" s="16">
-        <v>1</v>
-      </c>
-      <c r="K39" s="16">
-        <v>1</v>
-      </c>
-      <c r="L39" s="16">
-        <v>1</v>
-      </c>
-      <c r="M39" s="18">
-        <v>1</v>
-      </c>
-      <c r="N39" s="18">
-        <v>1</v>
-      </c>
-      <c r="O39" s="18">
-        <v>1</v>
-      </c>
-      <c r="P39" s="18">
-        <v>1</v>
-      </c>
-      <c r="Q39" s="18">
-        <v>1</v>
-      </c>
-      <c r="R39" s="18">
-        <v>1</v>
-      </c>
-      <c r="S39" s="18">
-        <v>1</v>
-      </c>
-      <c r="T39" s="18">
-        <v>1</v>
-      </c>
-      <c r="U39" s="18">
-        <v>1</v>
-      </c>
-      <c r="V39" s="5">
-        <v>1</v>
-      </c>
-      <c r="W39" s="26">
-        <f t="shared" si="0"/>
-        <v>20</v>
-      </c>
-    </row>
-    <row r="40" spans="1:23" ht="16">
-      <c r="A40" s="15" t="s">
-        <v>35</v>
       </c>
       <c r="B40" s="15"/>
       <c r="C40" s="15">
@@ -2899,47 +2864,81 @@
       <c r="E40" s="16">
         <v>1</v>
       </c>
-      <c r="F40" s="16"/>
-      <c r="G40" s="16"/>
-      <c r="H40" s="16"/>
-      <c r="I40" s="16"/>
-      <c r="J40" s="16"/>
-      <c r="K40" s="16"/>
-      <c r="L40" s="16"/>
-      <c r="M40" s="19"/>
-      <c r="N40" s="19"/>
-      <c r="O40" s="19"/>
-      <c r="P40" s="19"/>
-      <c r="Q40" s="19"/>
-      <c r="R40" s="19"/>
-      <c r="S40" s="19"/>
-      <c r="T40" s="27"/>
-      <c r="U40" s="27"/>
-      <c r="V40" s="5"/>
+      <c r="F40" s="16">
+        <v>1</v>
+      </c>
+      <c r="G40" s="16">
+        <v>1</v>
+      </c>
+      <c r="H40" s="16">
+        <v>1</v>
+      </c>
+      <c r="I40" s="16">
+        <v>1</v>
+      </c>
+      <c r="J40" s="16">
+        <v>1</v>
+      </c>
+      <c r="K40" s="16">
+        <v>1</v>
+      </c>
+      <c r="L40" s="16">
+        <v>1</v>
+      </c>
+      <c r="M40" s="18">
+        <v>1</v>
+      </c>
+      <c r="N40" s="18">
+        <v>1</v>
+      </c>
+      <c r="O40" s="18">
+        <v>1</v>
+      </c>
+      <c r="P40" s="18">
+        <v>1</v>
+      </c>
+      <c r="Q40" s="18">
+        <v>1</v>
+      </c>
+      <c r="R40" s="18">
+        <v>1</v>
+      </c>
+      <c r="S40" s="18">
+        <v>1</v>
+      </c>
+      <c r="T40" s="18">
+        <v>1</v>
+      </c>
+      <c r="U40" s="18">
+        <v>1</v>
+      </c>
+      <c r="V40" s="5">
+        <v>1</v>
+      </c>
       <c r="W40" s="26">
         <f t="shared" si="0"/>
-        <v>3</v>
+        <v>20</v>
       </c>
     </row>
     <row r="41" spans="1:23" ht="16">
       <c r="A41" s="15" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B41" s="15"/>
-      <c r="C41" s="15"/>
-      <c r="D41" s="15"/>
-      <c r="E41" s="16"/>
-      <c r="F41" s="15"/>
-      <c r="G41" s="15"/>
-      <c r="H41" s="16">
-        <v>1</v>
-      </c>
-      <c r="I41" s="16">
-        <v>1</v>
-      </c>
-      <c r="J41" s="16">
-        <v>1</v>
-      </c>
+      <c r="C41" s="15">
+        <v>1</v>
+      </c>
+      <c r="D41" s="16">
+        <v>1</v>
+      </c>
+      <c r="E41" s="16">
+        <v>1</v>
+      </c>
+      <c r="F41" s="16"/>
+      <c r="G41" s="16"/>
+      <c r="H41" s="16"/>
+      <c r="I41" s="16"/>
+      <c r="J41" s="16"/>
       <c r="K41" s="16"/>
       <c r="L41" s="16"/>
       <c r="M41" s="19"/>
@@ -2952,139 +2951,175 @@
       <c r="T41" s="27"/>
       <c r="U41" s="27"/>
       <c r="V41" s="5"/>
-      <c r="W41" s="7">
+      <c r="W41" s="26">
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
     </row>
     <row r="42" spans="1:23" ht="16">
-      <c r="A42" s="28" t="s">
+      <c r="A42" s="15" t="s">
+        <v>36</v>
+      </c>
+      <c r="B42" s="15"/>
+      <c r="C42" s="15"/>
+      <c r="D42" s="15"/>
+      <c r="E42" s="16"/>
+      <c r="F42" s="15"/>
+      <c r="G42" s="15"/>
+      <c r="H42" s="16">
+        <v>1</v>
+      </c>
+      <c r="I42" s="16">
+        <v>1</v>
+      </c>
+      <c r="J42" s="16">
+        <v>1</v>
+      </c>
+      <c r="K42" s="16"/>
+      <c r="L42" s="16"/>
+      <c r="M42" s="19"/>
+      <c r="N42" s="19"/>
+      <c r="O42" s="19"/>
+      <c r="P42" s="19"/>
+      <c r="Q42" s="19"/>
+      <c r="R42" s="19"/>
+      <c r="S42" s="19"/>
+      <c r="T42" s="27"/>
+      <c r="U42" s="27"/>
+      <c r="V42" s="5"/>
+      <c r="W42" s="7">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="43" spans="1:23" ht="16">
+      <c r="A43" s="28" t="s">
         <v>37</v>
       </c>
-      <c r="B42" s="28"/>
-      <c r="C42" s="29">
-        <v>1</v>
-      </c>
-      <c r="D42" s="28">
-        <v>1</v>
-      </c>
-      <c r="E42" s="30"/>
-      <c r="F42" s="30"/>
-      <c r="G42" s="30"/>
-      <c r="H42" s="30"/>
-      <c r="I42" s="30"/>
-      <c r="J42" s="30"/>
-      <c r="K42" s="31"/>
-      <c r="L42" s="31"/>
-      <c r="M42" s="32"/>
-      <c r="N42" s="32"/>
-      <c r="O42" s="32"/>
-      <c r="P42" s="32"/>
-      <c r="Q42" s="32"/>
-      <c r="R42" s="32"/>
-      <c r="S42" s="32"/>
-      <c r="T42" s="33"/>
-      <c r="U42" s="33"/>
-      <c r="V42" s="34"/>
-      <c r="W42" s="35">
+      <c r="B43" s="28"/>
+      <c r="C43" s="29">
+        <v>1</v>
+      </c>
+      <c r="D43" s="28">
+        <v>1</v>
+      </c>
+      <c r="E43" s="30"/>
+      <c r="F43" s="30"/>
+      <c r="G43" s="30"/>
+      <c r="H43" s="30"/>
+      <c r="I43" s="30"/>
+      <c r="J43" s="30"/>
+      <c r="K43" s="31"/>
+      <c r="L43" s="31"/>
+      <c r="M43" s="32"/>
+      <c r="N43" s="32"/>
+      <c r="O43" s="32"/>
+      <c r="P43" s="32"/>
+      <c r="Q43" s="32"/>
+      <c r="R43" s="32"/>
+      <c r="S43" s="32"/>
+      <c r="T43" s="33"/>
+      <c r="U43" s="33"/>
+      <c r="V43" s="34"/>
+      <c r="W43" s="35">
         <f t="shared" si="0"/>
         <v>2</v>
       </c>
     </row>
-    <row r="43" spans="1:23">
-      <c r="C43" s="15"/>
-      <c r="D43" s="15"/>
-      <c r="E43" s="15"/>
-      <c r="F43" s="15"/>
-      <c r="G43" s="15"/>
-      <c r="H43" s="16"/>
-      <c r="J43" s="16"/>
-      <c r="M43" s="36"/>
-    </row>
     <row r="44" spans="1:23">
-      <c r="A44" s="37" t="s">
+      <c r="C44" s="15"/>
+      <c r="D44" s="15"/>
+      <c r="E44" s="15"/>
+      <c r="F44" s="15"/>
+      <c r="G44" s="15"/>
+      <c r="H44" s="16"/>
+      <c r="J44" s="16"/>
+      <c r="M44" s="36"/>
+    </row>
+    <row r="45" spans="1:23">
+      <c r="A45" s="37" t="s">
         <v>38</v>
       </c>
-      <c r="B44" s="38"/>
-      <c r="C44" s="39">
-        <f>SUM(C3:C42)</f>
+      <c r="B45" s="38"/>
+      <c r="C45" s="39">
+        <f>SUM(C3:C43)</f>
         <v>18</v>
       </c>
-      <c r="D44" s="39">
-        <f>SUM(D3:D42)</f>
+      <c r="D45" s="39">
+        <f>SUM(D3:D43)</f>
         <v>16</v>
       </c>
-      <c r="E44" s="39">
-        <f>SUM(E3:E42)</f>
+      <c r="E45" s="39">
+        <f>SUM(E3:E43)</f>
         <v>16</v>
       </c>
-      <c r="F44" s="39">
-        <f t="shared" ref="F44:L44" si="1">SUM(F3:F42)</f>
+      <c r="F45" s="39">
+        <f>SUM(F3:F43)</f>
         <v>17</v>
       </c>
-      <c r="G44" s="39">
+      <c r="G45" s="39">
+        <f>SUM(G3:G43)</f>
+        <v>21</v>
+      </c>
+      <c r="H45" s="39">
+        <f>SUM(H3:H43)</f>
+        <v>25</v>
+      </c>
+      <c r="I45" s="39">
+        <f>SUM(I3:I43)</f>
+        <v>28</v>
+      </c>
+      <c r="J45" s="39">
+        <f>SUM(J3:J43)</f>
+        <v>30</v>
+      </c>
+      <c r="K45" s="39">
+        <f>SUM(K3:K43)</f>
+        <v>29</v>
+      </c>
+      <c r="L45" s="39">
+        <f>SUM(L3:L43)</f>
+        <v>26</v>
+      </c>
+      <c r="M45" s="40">
+        <f>SUM(M3:M44)</f>
+        <v>25</v>
+      </c>
+      <c r="N45" s="40">
+        <f t="shared" ref="N45:V45" si="1">SUM(N3:N44)</f>
+        <v>24</v>
+      </c>
+      <c r="O45" s="40">
         <f t="shared" si="1"/>
-        <v>21</v>
-      </c>
-      <c r="H44" s="39">
+        <v>24</v>
+      </c>
+      <c r="P45" s="40">
         <f t="shared" si="1"/>
-        <v>25</v>
-      </c>
-      <c r="I44" s="39">
+        <v>26</v>
+      </c>
+      <c r="Q45" s="40">
+        <f>SUM(Q3:Q44)</f>
+        <v>23</v>
+      </c>
+      <c r="R45" s="40">
+        <f t="shared" si="1"/>
+        <v>24.75</v>
+      </c>
+      <c r="S45" s="40">
+        <f t="shared" si="1"/>
+        <v>24.75</v>
+      </c>
+      <c r="T45" s="40">
+        <f t="shared" si="1"/>
+        <v>25.916666666666668</v>
+      </c>
+      <c r="U45" s="40">
+        <f t="shared" si="1"/>
+        <v>26.083333333333332</v>
+      </c>
+      <c r="V45" s="41">
         <f t="shared" si="1"/>
         <v>28</v>
-      </c>
-      <c r="J44" s="39">
-        <f t="shared" si="1"/>
-        <v>30</v>
-      </c>
-      <c r="K44" s="39">
-        <f t="shared" si="1"/>
-        <v>29</v>
-      </c>
-      <c r="L44" s="39">
-        <f t="shared" si="1"/>
-        <v>26</v>
-      </c>
-      <c r="M44" s="40">
-        <f>SUM(M3:M43)</f>
-        <v>25</v>
-      </c>
-      <c r="N44" s="40">
-        <f t="shared" ref="N44:V44" si="2">SUM(N3:N43)</f>
-        <v>24</v>
-      </c>
-      <c r="O44" s="40">
-        <f t="shared" si="2"/>
-        <v>24</v>
-      </c>
-      <c r="P44" s="40">
-        <f t="shared" si="2"/>
-        <v>26</v>
-      </c>
-      <c r="Q44" s="40">
-        <f>SUM(Q3:Q43)</f>
-        <v>23</v>
-      </c>
-      <c r="R44" s="40">
-        <f t="shared" si="2"/>
-        <v>24.75</v>
-      </c>
-      <c r="S44" s="40">
-        <f t="shared" si="2"/>
-        <v>24.75</v>
-      </c>
-      <c r="T44" s="40">
-        <f t="shared" si="2"/>
-        <v>25.916666666666668</v>
-      </c>
-      <c r="U44" s="40">
-        <f t="shared" si="2"/>
-        <v>26.083333333333332</v>
-      </c>
-      <c r="V44" s="41">
-        <f t="shared" si="2"/>
-        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>